<commit_message>
feat: default template to five exercises a day
Five exercises and sixteen sets is about an hour once rest is counted,
which is what a session actually looks like. Each day previously
generated six.

The sixth row of each day is kept but marked default = "no", so it
stays on the plan as a suggestion and doubles as a worked example of
that column. The build asserts five per day so the intent cannot drift.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/download/training-tracker-template.xlsx
+++ b/docs/download/training-tracker-template.xlsx
@@ -4829,6 +4829,11 @@
       <c r="E5">
         <v>0</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4997,6 +5002,11 @@
       <c r="E13">
         <v>0</v>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5122,6 +5132,11 @@
       </c>
       <c r="E19">
         <v>0</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add support for drop sets in workout log and UI
</commit_message>
<xml_diff>
--- a/docs/download/training-tracker-template.xlsx
+++ b/docs/download/training-tracker-template.xlsx
@@ -65,6 +65,11 @@
           <t xml:space="preserve">Group</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drop set</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>